<commit_message>
changed parameters in pandapower converter towards correct transformer parameters
</commit_message>
<xml_diff>
--- a/test_simbench.xlsx
+++ b/test_simbench.xlsx
@@ -1388,19 +1388,19 @@
     <t>0</t>
   </si>
   <si>
-    <t>88</t>
-  </si>
-  <si>
-    <t>70</t>
-  </si>
-  <si>
-    <t>81</t>
-  </si>
-  <si>
-    <t>92</t>
-  </si>
-  <si>
-    <t>54</t>
+    <t>47</t>
+  </si>
+  <si>
+    <t>43</t>
+  </si>
+  <si>
+    <t>49</t>
+  </si>
+  <si>
+    <t>73</t>
+  </si>
+  <si>
+    <t>14</t>
   </si>
   <si>
     <t>baseMVA</t>
@@ -10778,10 +10778,7 @@
         <v>208</v>
       </c>
       <c r="F2">
-        <v>0.1</v>
-      </c>
-      <c r="G2">
-        <v>0.1</v>
+        <v>0.00041</v>
       </c>
       <c r="H2" t="s">
         <v>320</v>
@@ -10831,10 +10828,7 @@
         <v>208</v>
       </c>
       <c r="F3">
-        <v>0.1</v>
-      </c>
-      <c r="G3">
-        <v>0.1</v>
+        <v>0.00041</v>
       </c>
       <c r="H3" t="s">
         <v>320</v>

</xml_diff>